<commit_message>
chore: run 2026-03-14 22:46 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_14_03_2026.xlsx
+++ b/logs/Consolidado_14_03_2026.xlsx
@@ -676,10 +676,10 @@
         <v>78</v>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -1744,12 +1744,12 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>3000724</t>
+          <t>6552595</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1786,12 +1786,12 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>6064105</t>
+          <t>6552595</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -12467,43 +12467,43 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>14/03/2026</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>Mango Nourishing Shampoo
 Champô Manga Nutritivo para Cabelo Seco</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D57" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
+      <c r="E57" s="7" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
         <is>
           <t>3018059</t>
         </is>
       </c>
-      <c r="H57" s="5" t="inlineStr">
+      <c r="H57" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -25721,12 +25721,12 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>3000724</t>
+          <t>6552595</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -25758,12 +25758,12 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>6064105</t>
+          <t>6552595</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -27179,38 +27179,38 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="7" t="inlineStr">
         <is>
           <t>Mango Nourishing Shampoo
 Champô Manga Nutritivo para Cabelo Seco</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C68" s="7" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="inlineStr">
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
         <is>
           <t>3018059</t>
         </is>
       </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
         </is>

</xml_diff>